<commit_message>
Add initial Jupyter notebook for Titanic dataset analysis
- Load Titanic dataset from CSV file into a pandas DataFrame
- Display the first few rows of the dataset
- Show rows with missing values in the 'body' column
- Calculate and display correlation of numeric features with survival
</commit_message>
<xml_diff>
--- a/outputs/missing_values.xlsx
+++ b/outputs/missing_values.xlsx
@@ -423,12 +423,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>transaction_id</t>
+          <t>expense_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>expense_date</t>
+          <t>date</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -448,12 +448,12 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>amount_krw</t>
+          <t>amount</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>approval_status</t>
+          <t>status</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -468,7 +468,7 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>source_filename</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
@@ -488,12 +488,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>People</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Meals</t>
+          <t>Food</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -517,115 +517,121 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>data\inbox\2026-01_hr_expenses.csv</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>1</v>
+          <t>2026-01_hr_expenses.csv</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>EX-202601-SA-06</t>
+          <t>EX-202601-MA-19</t>
         </is>
       </c>
       <c r="B3" s="1" t="n">
-        <v>46037</v>
+        <v>46028</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Client Events</t>
+          <t>출장비</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>COEX</t>
+          <t>Korean Air</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>2951000</v>
+        <v>802000</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>S123</t>
+          <t>M102</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>data\inbox\2026-01_sales_expenses.csv</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
-        <v>1</v>
+          <t>2026-01_marketing_expenses.xlsx</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>EX-202601-SA-08</t>
+          <t>EX-202601-OP-01</t>
         </is>
       </c>
       <c r="B4" s="1" t="n">
-        <v>46028</v>
+        <v>46037</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>L&amp;D</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>DataCloud Korea</t>
+          <t>Fast Campus</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>519000</v>
+        <v>1619000</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>S128</t>
+          <t>O142</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>data\inbox\2026-01_sales_expenses.csv</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
-        <v>1</v>
+          <t>2026-01_operations_expenses.xlsx</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>EX-202601-SA-19</t>
+          <t>EX-202601-SA-06</t>
         </is>
       </c>
       <c r="B5" s="1" t="n">
-        <v>46045</v>
+        <v>46037</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -634,16 +640,16 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Meals</t>
+          <t>Client Events</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Office Cafe</t>
+          <t>COEX</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>111000</v>
+        <v>2951000</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -652,45 +658,47 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>S135</t>
+          <t>S123</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
-          <t>data\inbox\2026-01_sales_expenses.csv</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>1</v>
+          <t>2026-01_sales_expenses.csv</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>EX-202602-MA-11</t>
+          <t>EX-202601-SA-08</t>
         </is>
       </c>
       <c r="B6" s="1" t="n">
-        <v>46057</v>
+        <v>46028</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Travel</t>
+          <t>SaaS</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Kakao T</t>
+          <t>DataCloud Korea</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>360000</v>
+        <v>519000</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -699,45 +707,47 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>M114</t>
+          <t>S128</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>data\inbox\2026-02_marketing_expenses.csv</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>2</v>
+          <t>2026-01_sales_expenses.csv</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>EX-202602-MA-22</t>
+          <t>EX-202601-SA-19</t>
         </is>
       </c>
       <c r="B7" s="1" t="n">
-        <v>46069</v>
+        <v>46045</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Travel</t>
+          <t>Meals</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Korean Air</t>
+          <t>Office Cafe</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>557000</v>
+        <v>111000</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -746,92 +756,96 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>M112</t>
+          <t>S135</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>data\inbox\2026-02_marketing_expenses.csv</t>
-        </is>
-      </c>
-      <c r="K7" t="n">
-        <v>2</v>
+          <t>2026-01_sales_expenses.csv</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>EX-202603-HR-16</t>
+          <t>EX-202602-MA-11</t>
         </is>
       </c>
       <c r="B8" s="1" t="n">
-        <v>46096</v>
+        <v>46057</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Meals</t>
+          <t>Business Travel</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Local Restaurant</t>
+          <t>Kakao T</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>104000</v>
+        <v>360000</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>H165</t>
+          <t>M114</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>data\inbox\2026-03_hr_expenses.csv</t>
-        </is>
-      </c>
-      <c r="K8" t="n">
-        <v>3</v>
+          <t>2026-02_marketing_expenses.csv</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>EX-202603-SA-02</t>
+          <t>EX-202602-MA-22</t>
         </is>
       </c>
       <c r="B9" s="1" t="n">
-        <v>46107</v>
+        <v>46069</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Meals</t>
+          <t>Business Travel</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Baemin</t>
+          <t>Korean Air</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>64000</v>
+        <v>557000</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -840,27 +854,29 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>S133</t>
+          <t>M112</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
-          <t>data\inbox\2026-03_sales_expenses.csv</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
-        <v>3</v>
+          <t>2026-02_marketing_expenses.csv</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>EX-202603-SA-15</t>
+          <t>EX-202602-SA-11</t>
         </is>
       </c>
       <c r="B10" s="1" t="n">
-        <v>46087</v>
+        <v>46078</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -869,16 +885,16 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Travel</t>
+          <t>SaaS</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Kakao T</t>
+          <t>DataCloud Korea</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>612000</v>
+        <v>373000</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -887,31 +903,33 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>S122</t>
+          <t>S133</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
-          <t>data\inbox\2026-03_sales_expenses.csv</t>
-        </is>
-      </c>
-      <c r="K10" t="n">
-        <v>3</v>
+          <t>2026-02_sales_expenses.xlsx</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>EX-202604-MA-03</t>
+          <t>EX-202602-SA-14</t>
         </is>
       </c>
       <c r="B11" s="1" t="n">
-        <v>46126</v>
+        <v>46059</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -921,152 +939,158 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Notion</t>
+          <t>DataCloud Korea</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>431000</v>
+        <v>452000</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>M117</t>
+          <t>S129</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>data\inbox\2026-04_marketing_expenses.csv</t>
-        </is>
-      </c>
-      <c r="K11" t="n">
-        <v>4</v>
+          <t>2026-02_sales_expenses.xlsx</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>EX-202604-MA-12</t>
+          <t>EX-202602-SA-15</t>
         </is>
       </c>
       <c r="B12" s="1" t="n">
-        <v>46128</v>
+        <v>46056</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Advertising</t>
+          <t>SaaS</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Kakao Business</t>
+          <t>Slack</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2364000</v>
+        <v>838000</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>M117</t>
+          <t>S125</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>data\inbox\2026-04_marketing_expenses.csv</t>
-        </is>
-      </c>
-      <c r="K12" t="n">
-        <v>4</v>
+          <t>2026-02_sales_expenses.xlsx</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>EX-202604-OP-15</t>
+          <t>EX-202603-HR-16</t>
         </is>
       </c>
       <c r="B13" s="1" t="n">
-        <v>46113</v>
+        <v>46096</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Food</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Coursera</t>
+          <t>Local Restaurant</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>769000</v>
+        <v>104000</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>O153</t>
+          <t>H165</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>data\inbox\2026-04_operations_expenses.csv</t>
-        </is>
-      </c>
-      <c r="K13" t="n">
-        <v>4</v>
+          <t>2026-03_hr_expenses.csv</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>EX-202605-HR-06</t>
+          <t>EX-202603-MA-14</t>
         </is>
       </c>
       <c r="B14" s="1" t="n">
-        <v>46149</v>
+        <v>46104</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Recruiting</t>
+          <t>Business Travel</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Saramin</t>
+          <t>Kakao T</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1652000</v>
+        <v>314000</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1075,45 +1099,47 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>H177</t>
+          <t>M102</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
-          <t>data\inbox\2026-05_hr_expenses.csv</t>
-        </is>
-      </c>
-      <c r="K14" t="n">
-        <v>5</v>
+          <t>2026-03_marketing_expenses.xlsx</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>EX-202605-SA-15</t>
+          <t>EX-202603-MA-15</t>
         </is>
       </c>
       <c r="B15" s="1" t="n">
-        <v>46159</v>
+        <v>46097</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>출장비</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Notion</t>
+          <t>Kakao T</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>393000</v>
+        <v>394000</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1122,92 +1148,96 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>S121</t>
+          <t>M112</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
-          <t>data\inbox\2026-05_sales_expenses.csv</t>
-        </is>
-      </c>
-      <c r="K15" t="n">
-        <v>5</v>
+          <t>2026-03_marketing_expenses.xlsx</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>EX-202606-MA-03</t>
+          <t>EX-202603-OP-01</t>
         </is>
       </c>
       <c r="B16" s="1" t="n">
-        <v>46177</v>
+        <v>46103</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Office Supplies</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Notion</t>
+          <t>Coupang Business</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>765000</v>
+        <v>224000</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>M110</t>
+          <t>O146</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
-          <t>data\inbox\2026-06_marketing_expenses.csv</t>
-        </is>
-      </c>
-      <c r="K16" t="n">
-        <v>6</v>
+          <t>2026-03_operations_expenses.xlsx</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>EX-202606-MA-18</t>
+          <t>EX-202603-OP-09</t>
         </is>
       </c>
       <c r="B17" s="1" t="n">
-        <v>46189</v>
+        <v>46104</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Training</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Notion</t>
+          <t>Coursera</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>371000</v>
+        <v>1090000</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1216,45 +1246,47 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>M113</t>
+          <t>O153</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
-          <t>data\inbox\2026-06_marketing_expenses.csv</t>
-        </is>
-      </c>
-      <c r="K17" t="n">
-        <v>6</v>
+          <t>2026-03_operations_expenses.xlsx</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>EX-202606-OP-15</t>
+          <t>EX-202603-SA-02</t>
         </is>
       </c>
       <c r="B18" s="1" t="n">
-        <v>46174</v>
+        <v>46107</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Meals</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Fast Campus</t>
+          <t>Baemin</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>1390000</v>
+        <v>64000</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1263,45 +1295,47 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>O146</t>
+          <t>S133</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
-          <t>data\inbox\2026-06_operations_expenses.csv</t>
-        </is>
-      </c>
-      <c r="K18" t="n">
-        <v>6</v>
+          <t>2026-03_sales_expenses.csv</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>EX-202601-MA-19</t>
+          <t>EX-202603-SA-15</t>
         </is>
       </c>
       <c r="B19" s="1" t="n">
-        <v>46028</v>
+        <v>46087</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Travel</t>
+          <t>출장비</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Korean Air</t>
+          <t>Kakao T</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>802000</v>
+        <v>612000</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1310,45 +1344,47 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>M102</t>
+          <t>S122</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
-          <t>data\inbox\2026-01_marketing_expenses.xlsx</t>
-        </is>
-      </c>
-      <c r="K19" t="n">
-        <v>1</v>
+          <t>2026-03_sales_expenses.csv</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>EX-202601-OP-01</t>
+          <t>EX-202604-HR-02</t>
         </is>
       </c>
       <c r="B20" s="1" t="n">
-        <v>46037</v>
+        <v>46137</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Recruiting</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Fast Campus</t>
+          <t>Wanted</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1619000</v>
+        <v>2151000</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1357,45 +1393,47 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>O142</t>
+          <t>H164</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
-          <t>data\inbox\2026-01_operations_expenses.xlsx</t>
-        </is>
-      </c>
-      <c r="K20" t="n">
-        <v>1</v>
+          <t>2026-04_hr_expenses.xlsx</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>EX-202602-SA-11</t>
+          <t>EX-202604-HR-04</t>
         </is>
       </c>
       <c r="B21" s="1" t="n">
-        <v>46078</v>
+        <v>46115</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>People</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>교육비</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>DataCloud Korea</t>
+          <t>Korea Management Institute</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>373000</v>
+        <v>1826000</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1404,45 +1442,47 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>S133</t>
+          <t>H161</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
-          <t>data\inbox\2026-02_sales_expenses.xlsx</t>
-        </is>
-      </c>
-      <c r="K21" t="n">
-        <v>2</v>
+          <t>2026-04_hr_expenses.xlsx</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>EX-202602-SA-14</t>
+          <t>EX-202604-HR-11</t>
         </is>
       </c>
       <c r="B22" s="1" t="n">
-        <v>46059</v>
+        <v>46119</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>People</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Training</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>DataCloud Korea</t>
+          <t>Fast Campus</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>452000</v>
+        <v>620000</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1451,31 +1491,33 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>S129</t>
+          <t>H169</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
-          <t>data\inbox\2026-02_sales_expenses.xlsx</t>
-        </is>
-      </c>
-      <c r="K22" t="n">
-        <v>2</v>
+          <t>2026-04_hr_expenses.xlsx</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>EX-202602-SA-15</t>
+          <t>EX-202604-MA-03</t>
         </is>
       </c>
       <c r="B23" s="1" t="n">
-        <v>46056</v>
+        <v>46126</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1485,11 +1527,11 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Slack</t>
+          <t>Notion</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>838000</v>
+        <v>431000</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1498,27 +1540,29 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>S125</t>
+          <t>M117</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
-          <t>data\inbox\2026-02_sales_expenses.xlsx</t>
-        </is>
-      </c>
-      <c r="K23" t="n">
-        <v>2</v>
+          <t>2026-04_marketing_expenses.csv</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EX-202603-MA-14</t>
+          <t>EX-202604-MA-12</t>
         </is>
       </c>
       <c r="B24" s="1" t="n">
-        <v>46104</v>
+        <v>46128</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1527,110 +1571,114 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Travel</t>
+          <t>Advertising</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Kakao T</t>
+          <t>Kakao Business</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>314000</v>
+        <v>2364000</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>M102</t>
+          <t>M117</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
-          <t>data\inbox\2026-03_marketing_expenses.xlsx</t>
-        </is>
-      </c>
-      <c r="K24" t="n">
-        <v>3</v>
+          <t>2026-04_marketing_expenses.csv</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>EX-202603-MA-15</t>
+          <t>EX-202604-OP-15</t>
         </is>
       </c>
       <c r="B25" s="1" t="n">
-        <v>46097</v>
+        <v>46113</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Travel</t>
+          <t>L&amp;D</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Kakao T</t>
+          <t>Coursera</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>394000</v>
+        <v>769000</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>M112</t>
+          <t>O153</t>
         </is>
       </c>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
-          <t>data\inbox\2026-03_marketing_expenses.xlsx</t>
-        </is>
-      </c>
-      <c r="K25" t="n">
-        <v>3</v>
+          <t>2026-04_operations_expenses.csv</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>EX-202603-OP-01</t>
+          <t>EX-202605-HR-06</t>
         </is>
       </c>
       <c r="B26" s="1" t="n">
-        <v>46103</v>
+        <v>46149</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>People</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Office Supplies</t>
+          <t>채용비</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Coupang Business</t>
+          <t>Saramin</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>224000</v>
+        <v>1652000</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1639,45 +1687,47 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>O146</t>
+          <t>H177</t>
         </is>
       </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
-          <t>data\inbox\2026-03_operations_expenses.xlsx</t>
-        </is>
-      </c>
-      <c r="K26" t="n">
-        <v>3</v>
+          <t>2026-05_hr_expenses.csv</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>EX-202603-OP-09</t>
+          <t>EX-202605-MA-24</t>
         </is>
       </c>
       <c r="B27" s="1" t="n">
-        <v>46104</v>
+        <v>46164</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Coursera</t>
+          <t>Notion</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>1090000</v>
+        <v>200000</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1686,46 +1736,46 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>O153</t>
+          <t>M115</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
-          <t>data\inbox\2026-03_operations_expenses.xlsx</t>
-        </is>
-      </c>
-      <c r="K27" t="n">
-        <v>3</v>
+          <t>2026-05_marketing_expenses.xlsx</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>EX-202604-HR-02</t>
+          <t>EX-202605-OP-06</t>
         </is>
       </c>
       <c r="B28" s="1" t="n">
-        <v>46137</v>
+        <v>46152</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Recruiting</t>
+          <t>Logistics</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Wanted</t>
-        </is>
-      </c>
-      <c r="F28" t="n">
-        <v>2151000</v>
-      </c>
+          <t>Quick Service Seoul</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1733,139 +1783,149 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>H164</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr"/>
+          <t>O148</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Logistics expense</t>
+        </is>
+      </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>data\inbox\2026-04_hr_expenses.xlsx</t>
-        </is>
-      </c>
-      <c r="K28" t="n">
-        <v>4</v>
+          <t>2026-05_operations_expenses.xlsx</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>EX-202604-HR-04</t>
+          <t>EX-202605-OP-15</t>
         </is>
       </c>
       <c r="B29" s="1" t="n">
-        <v>46115</v>
+        <v>46153</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>SaaS</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Korea Management Institute</t>
+          <t>DataCloud Korea</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>1826000</v>
+        <v>761000</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>H161</t>
+          <t>O157</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
-          <t>data\inbox\2026-04_hr_expenses.xlsx</t>
-        </is>
-      </c>
-      <c r="K29" t="n">
-        <v>4</v>
+          <t>2026-05_operations_expenses.xlsx</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>EX-202604-HR-11</t>
+          <t>EX-202605-SA-15</t>
         </is>
       </c>
       <c r="B30" s="1" t="n">
-        <v>46119</v>
+        <v>46159</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Fast Campus</t>
+          <t>Notion</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>620000</v>
+        <v>393000</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>H169</t>
+          <t>S121</t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
-          <t>data\inbox\2026-04_hr_expenses.xlsx</t>
-        </is>
-      </c>
-      <c r="K30" t="n">
-        <v>4</v>
+          <t>2026-05_sales_expenses.csv</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>EX-202605-MA-24</t>
+          <t>EX-202606-HR-15</t>
         </is>
       </c>
       <c r="B31" s="1" t="n">
-        <v>46164</v>
+        <v>46186</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>People</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>Meals</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Notion</t>
+          <t>Office Cafe</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>200000</v>
+        <v>57000</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1874,44 +1934,48 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>M115</t>
+          <t>H168</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
-          <t>data\inbox\2026-05_marketing_expenses.xlsx</t>
-        </is>
-      </c>
-      <c r="K31" t="n">
-        <v>5</v>
+          <t>2026-06_hr_expenses.xlsx</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>EX-202605-OP-06</t>
+          <t>EX-202606-MA-03</t>
         </is>
       </c>
       <c r="B32" s="1" t="n">
-        <v>46152</v>
+        <v>46177</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Logistics</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Quick Service Seoul</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr"/>
+          <t>Notion</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>765000</v>
+      </c>
       <c r="G32" t="inlineStr">
         <is>
           <t>Approved</t>
@@ -1919,35 +1983,33 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>O148</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>Logistics expense</t>
-        </is>
-      </c>
+          <t>M110</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr">
         <is>
-          <t>data\inbox\2026-05_operations_expenses.xlsx</t>
-        </is>
-      </c>
-      <c r="K32" t="n">
-        <v>5</v>
+          <t>2026-06_marketing_expenses.csv</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>EX-202605-OP-15</t>
+          <t>EX-202606-MA-18</t>
         </is>
       </c>
       <c r="B33" s="1" t="n">
-        <v>46153</v>
+        <v>46189</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1957,58 +2019,60 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>DataCloud Korea</t>
+          <t>Notion</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>761000</v>
+        <v>371000</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>O157</t>
+          <t>M113</t>
         </is>
       </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
-          <t>data\inbox\2026-05_operations_expenses.xlsx</t>
-        </is>
-      </c>
-      <c r="K33" t="n">
-        <v>5</v>
+          <t>2026-06_marketing_expenses.csv</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>EX-202606-HR-15</t>
+          <t>EX-202606-OP-15</t>
         </is>
       </c>
       <c r="B34" s="1" t="n">
-        <v>46186</v>
+        <v>46174</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Meals</t>
+          <t>Training</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Office Cafe</t>
+          <t>Fast Campus</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>57000</v>
+        <v>1390000</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -2017,17 +2081,19 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>H168</t>
+          <t>O146</t>
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
-          <t>data\inbox\2026-06_hr_expenses.xlsx</t>
-        </is>
-      </c>
-      <c r="K34" t="n">
-        <v>6</v>
+          <t>2026-06_operations_expenses.csv</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -2070,11 +2136,13 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>data\inbox\2026-06_sales_expenses.xlsx</t>
-        </is>
-      </c>
-      <c r="K35" t="n">
-        <v>6</v>
+          <t>2026-06_sales_expenses.xlsx</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>